<commit_message>
Consolidate Software Engineering syllabus from 18 to 14 units
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GziQKc7swEifeixDXPPfmU
</commit_message>
<xml_diff>
--- a/Course_Blueprint_for_Software_Engineering.xlsx
+++ b/Course_Blueprint_for_Software_Engineering.xlsx
@@ -713,7 +713,7 @@
       </c>
       <c r="B14" s="18" t="inlineStr">
         <is>
-          <t>Software Process Models</t>
+          <t>Software Process Models &amp; Agile Methods</t>
         </is>
       </c>
       <c r="C14" s="18" t="inlineStr">
@@ -854,14 +854,8 @@
       </c>
     </row>
     <row r="24" s="16">
-      <c r="A24" s="18" t="n">
-        <v>3</v>
-      </c>
-      <c r="B24" s="18" t="inlineStr">
-        <is>
-          <t>Agile Methods &amp; Team Practices</t>
-        </is>
-      </c>
+      <c r="A24" s="18" t="n"/>
+      <c r="B24" s="18" t="n"/>
       <c r="C24" s="18" t="inlineStr">
         <is>
           <t>The Agile Manifesto and Its Principles</t>
@@ -1015,7 +1009,7 @@
     </row>
     <row r="35" s="16">
       <c r="A35" s="18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
@@ -1189,7 +1183,7 @@
     </row>
     <row r="47" s="16">
       <c r="A47" s="18" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
@@ -1349,7 +1343,7 @@
     </row>
     <row r="58" s="16">
       <c r="A58" s="18" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B58" s="18" t="inlineStr">
         <is>
@@ -1523,7 +1517,7 @@
     </row>
     <row r="70" s="16">
       <c r="A70" s="18" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B70" s="18" t="inlineStr">
         <is>
@@ -1697,7 +1691,7 @@
     </row>
     <row r="82" s="16">
       <c r="A82" s="18" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B82" s="18" t="inlineStr">
         <is>
@@ -1871,11 +1865,11 @@
     </row>
     <row r="94" s="16">
       <c r="A94" s="18" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B94" s="18" t="inlineStr">
         <is>
-          <t>Clean Code &amp; Refactoring</t>
+          <t>Clean Code, Refactoring &amp; Software Evolution</t>
         </is>
       </c>
       <c r="C94" s="18" t="inlineStr">
@@ -2030,22 +2024,16 @@
       </c>
     </row>
     <row r="105" s="16">
-      <c r="A105" s="18" t="n">
-        <v>10</v>
-      </c>
-      <c r="B105" s="18" t="inlineStr">
-        <is>
-          <t>Version Control &amp; Collaboration</t>
-        </is>
-      </c>
+      <c r="A105" s="18" t="n"/>
+      <c r="B105" s="18" t="n"/>
       <c r="C105" s="18" t="inlineStr">
         <is>
-          <t>Why Version Control?</t>
+          <t>Why Software Changes</t>
         </is>
       </c>
       <c r="D105" s="18" t="inlineStr">
         <is>
-          <t>History, collaboration, backup, accountability, centralized vs distributed</t>
+          <t>Lehman's laws, corrective, adaptive, perfective, preventive maintenance</t>
         </is>
       </c>
     </row>
@@ -2054,12 +2042,12 @@
       <c r="B106" s="18" t="n"/>
       <c r="C106" s="18" t="inlineStr">
         <is>
-          <t>Git Fundamentals</t>
+          <t>The Cost of Maintenance</t>
         </is>
       </c>
       <c r="D106" s="18" t="inlineStr">
         <is>
-          <t>Repository, working tree, staging area, commits, snapshots</t>
+          <t>Maintenance share of lifecycle cost, factors affecting maintainability</t>
         </is>
       </c>
     </row>
@@ -2068,12 +2056,12 @@
       <c r="B107" s="18" t="n"/>
       <c r="C107" s="18" t="inlineStr">
         <is>
-          <t>Commits, History and Good Commit Messages</t>
+          <t>Change Impact Analysis</t>
         </is>
       </c>
       <c r="D107" s="18" t="inlineStr">
         <is>
-          <t>Atomic commits, log, diff, message conventions</t>
+          <t>Dependencies, ripple effects, risk of change</t>
         </is>
       </c>
     </row>
@@ -2082,12 +2070,12 @@
       <c r="B108" s="18" t="n"/>
       <c r="C108" s="18" t="inlineStr">
         <is>
-          <t>Branching and Merging</t>
+          <t>Reverse Engineering and Program Comprehension</t>
         </is>
       </c>
       <c r="D108" s="18" t="inlineStr">
         <is>
-          <t>Branches, fast-forward, merge commits, conflicts</t>
+          <t>Understanding unfamiliar systems, tools, documentation recovery</t>
         </is>
       </c>
     </row>
@@ -2096,12 +2084,12 @@
       <c r="B109" s="18" t="n"/>
       <c r="C109" s="18" t="inlineStr">
         <is>
-          <t>Resolving Merge Conflicts</t>
+          <t>Reengineering and Modernization</t>
         </is>
       </c>
       <c r="D109" s="18" t="inlineStr">
         <is>
-          <t>Conflict markers, resolution strategies, preventing conflicts</t>
+          <t>Rewrite vs refactor, strangler pattern, migration planning</t>
         </is>
       </c>
     </row>
@@ -2110,12 +2098,12 @@
       <c r="B110" s="18" t="n"/>
       <c r="C110" s="18" t="inlineStr">
         <is>
-          <t>Remote Repositories and Collaboration</t>
+          <t>Software Reuse</t>
         </is>
       </c>
       <c r="D110" s="18" t="inlineStr">
         <is>
-          <t>Clone, fetch, pull, push, forks, upstream</t>
+          <t>Libraries, frameworks, components, reuse benefits and costs</t>
         </is>
       </c>
     </row>
@@ -2124,12 +2112,12 @@
       <c r="B111" s="18" t="n"/>
       <c r="C111" s="18" t="inlineStr">
         <is>
-          <t>Branching Strategies</t>
+          <t>Software Documentation</t>
         </is>
       </c>
       <c r="D111" s="18" t="inlineStr">
         <is>
-          <t>Git Flow, GitHub Flow, trunk-based development</t>
+          <t>README, API docs, runbooks, living documentation</t>
         </is>
       </c>
     </row>
@@ -2138,12 +2126,12 @@
       <c r="B112" s="18" t="n"/>
       <c r="C112" s="18" t="inlineStr">
         <is>
-          <t>Pull Requests and Code Review Workflow</t>
+          <t>Configuration Management and Release Management</t>
         </is>
       </c>
       <c r="D112" s="18" t="inlineStr">
         <is>
-          <t>Small PRs, reviewers, feedback, approvals, merge policies</t>
+          <t>Baselines, change control boards, release planning</t>
         </is>
       </c>
     </row>
@@ -2152,26 +2140,32 @@
       <c r="B113" s="18" t="n"/>
       <c r="C113" s="18" t="inlineStr">
         <is>
-          <t>Rebasing, Cherry-Picking and Rewriting History</t>
+          <t>End of Life and Software Sustainability</t>
         </is>
       </c>
       <c r="D113" s="18" t="inlineStr">
         <is>
-          <t>Rebase vs merge, interactive rebase, reflog, safe practices</t>
+          <t>Deprecation, sunsetting, long-term support, green software</t>
         </is>
       </c>
     </row>
     <row r="114" s="16">
-      <c r="A114" s="18" t="n"/>
-      <c r="B114" s="18" t="n"/>
+      <c r="A114" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="B114" s="18" t="inlineStr">
+        <is>
+          <t>Version Control, Build &amp; DevOps</t>
+        </is>
+      </c>
       <c r="C114" s="18" t="inlineStr">
         <is>
-          <t>Tags, Releases and Semantic Versioning</t>
+          <t>Why Version Control?</t>
         </is>
       </c>
       <c r="D114" s="18" t="inlineStr">
         <is>
-          <t>Version numbers, release notes, changelogs, backward compatibility</t>
+          <t>History, collaboration, backup, accountability, centralized vs distributed</t>
         </is>
       </c>
     </row>
@@ -2180,12 +2174,12 @@
       <c r="B115" s="18" t="n"/>
       <c r="C115" s="18" t="inlineStr">
         <is>
-          <t>Issue Tracking and Project Boards</t>
+          <t>Git Fundamentals</t>
         </is>
       </c>
       <c r="D115" s="18" t="inlineStr">
         <is>
-          <t>Issues, labels, milestones, linking work to code</t>
+          <t>Repository, working tree, staging area, commits, snapshots</t>
         </is>
       </c>
     </row>
@@ -2194,32 +2188,26 @@
       <c r="B116" s="18" t="n"/>
       <c r="C116" s="18" t="inlineStr">
         <is>
-          <t>Open-Source Collaboration</t>
+          <t>Commits, History and Good Commit Messages</t>
         </is>
       </c>
       <c r="D116" s="18" t="inlineStr">
         <is>
-          <t>Contributing guidelines, licenses, community etiquette, first contributions</t>
+          <t>Atomic commits, log, diff, message conventions</t>
         </is>
       </c>
     </row>
     <row r="117" s="16">
-      <c r="A117" s="18" t="n">
-        <v>11</v>
-      </c>
-      <c r="B117" s="18" t="inlineStr">
-        <is>
-          <t>Software Testing Fundamentals</t>
-        </is>
-      </c>
+      <c r="A117" s="18" t="n"/>
+      <c r="B117" s="18" t="n"/>
       <c r="C117" s="18" t="inlineStr">
         <is>
-          <t>Why Test Software?</t>
+          <t>Branching and Merging</t>
         </is>
       </c>
       <c r="D117" s="18" t="inlineStr">
         <is>
-          <t>Bugs, failures, faults, cost of defects, testing limits</t>
+          <t>Branches, fast-forward, merge commits, conflicts</t>
         </is>
       </c>
     </row>
@@ -2228,12 +2216,12 @@
       <c r="B118" s="18" t="n"/>
       <c r="C118" s="18" t="inlineStr">
         <is>
-          <t>Testing Terminology and the Test Pyramid</t>
+          <t>Resolving Merge Conflicts</t>
         </is>
       </c>
       <c r="D118" s="18" t="inlineStr">
         <is>
-          <t>Error, fault, failure, unit, integration, system, acceptance</t>
+          <t>Conflict markers, resolution strategies, preventing conflicts</t>
         </is>
       </c>
     </row>
@@ -2242,12 +2230,12 @@
       <c r="B119" s="18" t="n"/>
       <c r="C119" s="18" t="inlineStr">
         <is>
-          <t>Unit Testing</t>
+          <t>Remote Repositories and Collaboration</t>
         </is>
       </c>
       <c r="D119" s="18" t="inlineStr">
         <is>
-          <t>Test cases, assertions, test frameworks, isolation, arrange-act-assert</t>
+          <t>Clone, fetch, pull, push, forks, upstream</t>
         </is>
       </c>
     </row>
@@ -2256,12 +2244,12 @@
       <c r="B120" s="18" t="n"/>
       <c r="C120" s="18" t="inlineStr">
         <is>
-          <t>Test Design: Equivalence Partitioning and Boundary Value Analysis</t>
+          <t>Branching Strategies</t>
         </is>
       </c>
       <c r="D120" s="18" t="inlineStr">
         <is>
-          <t>Input classes, boundaries, systematic case selection</t>
+          <t>Git Flow, GitHub Flow, trunk-based development</t>
         </is>
       </c>
     </row>
@@ -2270,12 +2258,12 @@
       <c r="B121" s="18" t="n"/>
       <c r="C121" s="18" t="inlineStr">
         <is>
-          <t>Test Design: Decision Tables and State-Based Testing</t>
+          <t>Pull Requests and Code Review Workflow</t>
         </is>
       </c>
       <c r="D121" s="18" t="inlineStr">
         <is>
-          <t>Combinations of conditions, state transitions</t>
+          <t>Small PRs, reviewers, feedback, approvals, merge policies</t>
         </is>
       </c>
     </row>
@@ -2284,12 +2272,12 @@
       <c r="B122" s="18" t="n"/>
       <c r="C122" s="18" t="inlineStr">
         <is>
-          <t>White-Box Testing and Code Coverage</t>
+          <t>Rebasing, Cherry-Picking and Rewriting History</t>
         </is>
       </c>
       <c r="D122" s="18" t="inlineStr">
         <is>
-          <t>Statement, branch, condition coverage, limits of coverage</t>
+          <t>Rebase vs merge, interactive rebase, reflog, safe practices</t>
         </is>
       </c>
     </row>
@@ -2298,12 +2286,12 @@
       <c r="B123" s="18" t="n"/>
       <c r="C123" s="18" t="inlineStr">
         <is>
-          <t>Test Doubles: Stubs, Mocks and Fakes</t>
+          <t>Tags, Releases and Semantic Versioning</t>
         </is>
       </c>
       <c r="D123" s="18" t="inlineStr">
         <is>
-          <t>Isolating dependencies, mocking frameworks, over-mocking</t>
+          <t>Version numbers, release notes, changelogs, backward compatibility</t>
         </is>
       </c>
     </row>
@@ -2312,12 +2300,12 @@
       <c r="B124" s="18" t="n"/>
       <c r="C124" s="18" t="inlineStr">
         <is>
-          <t>Test-Driven Development</t>
+          <t>Issue Tracking and Project Boards</t>
         </is>
       </c>
       <c r="D124" s="18" t="inlineStr">
         <is>
-          <t>Red-green-refactor, design through tests, benefits and limits</t>
+          <t>Issues, labels, milestones, linking work to code</t>
         </is>
       </c>
     </row>
@@ -2326,12 +2314,12 @@
       <c r="B125" s="18" t="n"/>
       <c r="C125" s="18" t="inlineStr">
         <is>
-          <t>Behaviour-Driven Development</t>
+          <t>Open-Source Collaboration</t>
         </is>
       </c>
       <c r="D125" s="18" t="inlineStr">
         <is>
-          <t>Given-When-Then, executable specifications, shared language</t>
+          <t>Contributing guidelines, licenses, community etiquette, first contributions</t>
         </is>
       </c>
     </row>
@@ -2340,12 +2328,12 @@
       <c r="B126" s="18" t="n"/>
       <c r="C126" s="18" t="inlineStr">
         <is>
-          <t>Integration and System Testing</t>
+          <t>From Source Code to Deployable Software</t>
         </is>
       </c>
       <c r="D126" s="18" t="inlineStr">
         <is>
-          <t>Interfaces, test environments, end-to-end flows</t>
+          <t>Compilation, dependencies, packaging, artifacts</t>
         </is>
       </c>
     </row>
@@ -2354,12 +2342,12 @@
       <c r="B127" s="18" t="n"/>
       <c r="C127" s="18" t="inlineStr">
         <is>
-          <t>Regression Testing and Test Automation</t>
+          <t>Build Tools and Dependency Management</t>
         </is>
       </c>
       <c r="D127" s="18" t="inlineStr">
         <is>
-          <t>Re-running tests, automation strategy, flaky tests</t>
+          <t>Package managers, lock files, reproducible builds, dependency hell</t>
         </is>
       </c>
     </row>
@@ -2368,12 +2356,12 @@
       <c r="B128" s="18" t="n"/>
       <c r="C128" s="18" t="inlineStr">
         <is>
-          <t>Acceptance, Exploratory and Usability Testing</t>
+          <t>Continuous Integration</t>
         </is>
       </c>
       <c r="D128" s="18" t="inlineStr">
         <is>
-          <t>Customer validation, session-based exploration, user feedback</t>
+          <t>Frequent integration, automated builds, fast feedback, build breaks</t>
         </is>
       </c>
     </row>
@@ -2382,12 +2370,12 @@
       <c r="B129" s="18" t="n"/>
       <c r="C129" s="18" t="inlineStr">
         <is>
-          <t>Non-Functional Testing</t>
+          <t>Continuous Delivery and Deployment</t>
         </is>
       </c>
       <c r="D129" s="18" t="inlineStr">
         <is>
-          <t>Performance, load, stress, security, accessibility testing</t>
+          <t>Pipelines, release automation, deployment strategies</t>
         </is>
       </c>
     </row>
@@ -2396,12 +2384,12 @@
       <c r="B130" s="18" t="n"/>
       <c r="C130" s="18" t="inlineStr">
         <is>
-          <t>Debugging Systematically</t>
+          <t>Environments and Configuration Management</t>
         </is>
       </c>
       <c r="D130" s="18" t="inlineStr">
         <is>
-          <t>Reproducing bugs, hypothesis testing, debuggers, logging, bisecting</t>
+          <t>Dev, test, staging, production, configuration vs code, secrets</t>
         </is>
       </c>
     </row>
@@ -2410,32 +2398,26 @@
       <c r="B131" s="18" t="n"/>
       <c r="C131" s="18" t="inlineStr">
         <is>
-          <t>Writing Good Bug Reports</t>
+          <t>Containers for Developers</t>
         </is>
       </c>
       <c r="D131" s="18" t="inlineStr">
         <is>
-          <t>Steps to reproduce, expected vs actual, severity, triage</t>
+          <t>Images, containers, Docker basics, portable environments</t>
         </is>
       </c>
     </row>
     <row r="132" s="16">
-      <c r="A132" s="18" t="n">
-        <v>12</v>
-      </c>
-      <c r="B132" s="18" t="inlineStr">
-        <is>
-          <t>Quality Assurance &amp; Verification</t>
-        </is>
-      </c>
+      <c r="A132" s="18" t="n"/>
+      <c r="B132" s="18" t="n"/>
       <c r="C132" s="18" t="inlineStr">
         <is>
-          <t>Software Quality: Definitions and Models</t>
+          <t>Infrastructure as Code</t>
         </is>
       </c>
       <c r="D132" s="18" t="inlineStr">
         <is>
-          <t>Quality attributes, ISO/IEC 25010, quality in use</t>
+          <t>Declarative infrastructure, repeatability, version-controlled environments</t>
         </is>
       </c>
     </row>
@@ -2444,12 +2426,12 @@
       <c r="B133" s="18" t="n"/>
       <c r="C133" s="18" t="inlineStr">
         <is>
-          <t>Quality Assurance vs Quality Control</t>
+          <t>Release Strategies</t>
         </is>
       </c>
       <c r="D133" s="18" t="inlineStr">
         <is>
-          <t>Process focus vs product focus, QA activities</t>
+          <t>Blue-green, canary, feature flags, rollbacks</t>
         </is>
       </c>
     </row>
@@ -2458,12 +2440,12 @@
       <c r="B134" s="18" t="n"/>
       <c r="C134" s="18" t="inlineStr">
         <is>
-          <t>Code Reviews and Inspections</t>
+          <t>Monitoring, Logging and Observability</t>
         </is>
       </c>
       <c r="D134" s="18" t="inlineStr">
         <is>
-          <t>Walkthroughs, formal inspection, checklists, review etiquette</t>
+          <t>Logs, metrics, traces, alerts, dashboards</t>
         </is>
       </c>
     </row>
@@ -2472,12 +2454,12 @@
       <c r="B135" s="18" t="n"/>
       <c r="C135" s="18" t="inlineStr">
         <is>
-          <t>Static Analysis and Linting</t>
+          <t>Incident Response and Postmortems</t>
         </is>
       </c>
       <c r="D135" s="18" t="inlineStr">
         <is>
-          <t>Automated checks, bug patterns, false positives</t>
+          <t>On-call, severity levels, blameless postmortems, learning culture</t>
         </is>
       </c>
     </row>
@@ -2486,26 +2468,32 @@
       <c r="B136" s="18" t="n"/>
       <c r="C136" s="18" t="inlineStr">
         <is>
-          <t>Software Metrics</t>
+          <t>The DevOps Culture</t>
         </is>
       </c>
       <c r="D136" s="18" t="inlineStr">
         <is>
-          <t>Lines of code, cyclomatic complexity, coupling metrics, defect density</t>
+          <t>Shared ownership, automation, measurement, DORA metrics</t>
         </is>
       </c>
     </row>
     <row r="137" s="16">
-      <c r="A137" s="18" t="n"/>
-      <c r="B137" s="18" t="n"/>
+      <c r="A137" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="B137" s="18" t="inlineStr">
+        <is>
+          <t>Software Testing Fundamentals</t>
+        </is>
+      </c>
       <c r="C137" s="18" t="inlineStr">
         <is>
-          <t>Defect Management and Root-Cause Analysis</t>
+          <t>Why Test Software?</t>
         </is>
       </c>
       <c r="D137" s="18" t="inlineStr">
         <is>
-          <t>Defect lifecycle, classification, five whys, prevention</t>
+          <t>Bugs, failures, faults, cost of defects, testing limits</t>
         </is>
       </c>
     </row>
@@ -2514,12 +2502,12 @@
       <c r="B138" s="18" t="n"/>
       <c r="C138" s="18" t="inlineStr">
         <is>
-          <t>Reliability and Availability Basics</t>
+          <t>Testing Terminology and the Test Pyramid</t>
         </is>
       </c>
       <c r="D138" s="18" t="inlineStr">
         <is>
-          <t>MTBF, MTTR, failure rates, fault tolerance</t>
+          <t>Error, fault, failure, unit, integration, system, acceptance</t>
         </is>
       </c>
     </row>
@@ -2528,12 +2516,12 @@
       <c r="B139" s="18" t="n"/>
       <c r="C139" s="18" t="inlineStr">
         <is>
-          <t>Formal Specification and Verification: An Introduction</t>
+          <t>Unit Testing</t>
         </is>
       </c>
       <c r="D139" s="18" t="inlineStr">
         <is>
-          <t>Invariants, assertions, model checking, when formal methods pay off</t>
+          <t>Test cases, assertions, test frameworks, isolation, arrange-act-assert</t>
         </is>
       </c>
     </row>
@@ -2542,12 +2530,12 @@
       <c r="B140" s="18" t="n"/>
       <c r="C140" s="18" t="inlineStr">
         <is>
-          <t>Safety-Critical Software</t>
+          <t>Test Design: Equivalence Partitioning and Boundary Value Analysis</t>
         </is>
       </c>
       <c r="D140" s="18" t="inlineStr">
         <is>
-          <t>Hazard analysis, standards, certification, case studies</t>
+          <t>Input classes, boundaries, systematic case selection</t>
         </is>
       </c>
     </row>
@@ -2556,32 +2544,26 @@
       <c r="B141" s="18" t="n"/>
       <c r="C141" s="18" t="inlineStr">
         <is>
-          <t>Learning from Failures</t>
+          <t>Test Design: Decision Tables and State-Based Testing</t>
         </is>
       </c>
       <c r="D141" s="18" t="inlineStr">
         <is>
-          <t>Therac-25, Ariane 5, Knight Capital, post-mortem analysis</t>
+          <t>Combinations of conditions, state transitions</t>
         </is>
       </c>
     </row>
     <row r="142" s="16">
-      <c r="A142" s="18" t="n">
-        <v>13</v>
-      </c>
-      <c r="B142" s="18" t="inlineStr">
-        <is>
-          <t>Build, Release &amp; DevOps</t>
-        </is>
-      </c>
+      <c r="A142" s="18" t="n"/>
+      <c r="B142" s="18" t="n"/>
       <c r="C142" s="18" t="inlineStr">
         <is>
-          <t>From Source Code to Deployable Software</t>
+          <t>White-Box Testing and Code Coverage</t>
         </is>
       </c>
       <c r="D142" s="18" t="inlineStr">
         <is>
-          <t>Compilation, dependencies, packaging, artifacts</t>
+          <t>Statement, branch, condition coverage, limits of coverage</t>
         </is>
       </c>
     </row>
@@ -2590,12 +2572,12 @@
       <c r="B143" s="18" t="n"/>
       <c r="C143" s="18" t="inlineStr">
         <is>
-          <t>Build Tools and Dependency Management</t>
+          <t>Test Doubles: Stubs, Mocks and Fakes</t>
         </is>
       </c>
       <c r="D143" s="18" t="inlineStr">
         <is>
-          <t>Package managers, lock files, reproducible builds, dependency hell</t>
+          <t>Isolating dependencies, mocking frameworks, over-mocking</t>
         </is>
       </c>
     </row>
@@ -2604,12 +2586,12 @@
       <c r="B144" s="18" t="n"/>
       <c r="C144" s="18" t="inlineStr">
         <is>
-          <t>Continuous Integration</t>
+          <t>Test-Driven Development</t>
         </is>
       </c>
       <c r="D144" s="18" t="inlineStr">
         <is>
-          <t>Frequent integration, automated builds, fast feedback, build breaks</t>
+          <t>Red-green-refactor, design through tests, benefits and limits</t>
         </is>
       </c>
     </row>
@@ -2618,12 +2600,12 @@
       <c r="B145" s="18" t="n"/>
       <c r="C145" s="18" t="inlineStr">
         <is>
-          <t>Continuous Delivery and Deployment</t>
+          <t>Behaviour-Driven Development</t>
         </is>
       </c>
       <c r="D145" s="18" t="inlineStr">
         <is>
-          <t>Pipelines, release automation, deployment strategies</t>
+          <t>Given-When-Then, executable specifications, shared language</t>
         </is>
       </c>
     </row>
@@ -2632,12 +2614,12 @@
       <c r="B146" s="18" t="n"/>
       <c r="C146" s="18" t="inlineStr">
         <is>
-          <t>Environments and Configuration Management</t>
+          <t>Integration and System Testing</t>
         </is>
       </c>
       <c r="D146" s="18" t="inlineStr">
         <is>
-          <t>Dev, test, staging, production, configuration vs code, secrets</t>
+          <t>Interfaces, test environments, end-to-end flows</t>
         </is>
       </c>
     </row>
@@ -2646,12 +2628,12 @@
       <c r="B147" s="18" t="n"/>
       <c r="C147" s="18" t="inlineStr">
         <is>
-          <t>Containers for Developers</t>
+          <t>Regression Testing and Test Automation</t>
         </is>
       </c>
       <c r="D147" s="18" t="inlineStr">
         <is>
-          <t>Images, containers, Docker basics, portable environments</t>
+          <t>Re-running tests, automation strategy, flaky tests</t>
         </is>
       </c>
     </row>
@@ -2660,12 +2642,12 @@
       <c r="B148" s="18" t="n"/>
       <c r="C148" s="18" t="inlineStr">
         <is>
-          <t>Infrastructure as Code</t>
+          <t>Acceptance, Exploratory and Usability Testing</t>
         </is>
       </c>
       <c r="D148" s="18" t="inlineStr">
         <is>
-          <t>Declarative infrastructure, repeatability, version-controlled environments</t>
+          <t>Customer validation, session-based exploration, user feedback</t>
         </is>
       </c>
     </row>
@@ -2674,12 +2656,12 @@
       <c r="B149" s="18" t="n"/>
       <c r="C149" s="18" t="inlineStr">
         <is>
-          <t>Release Strategies</t>
+          <t>Non-Functional Testing</t>
         </is>
       </c>
       <c r="D149" s="18" t="inlineStr">
         <is>
-          <t>Blue-green, canary, feature flags, rollbacks</t>
+          <t>Performance, load, stress, security, accessibility testing</t>
         </is>
       </c>
     </row>
@@ -2688,12 +2670,12 @@
       <c r="B150" s="18" t="n"/>
       <c r="C150" s="18" t="inlineStr">
         <is>
-          <t>Monitoring, Logging and Observability</t>
+          <t>Debugging Systematically</t>
         </is>
       </c>
       <c r="D150" s="18" t="inlineStr">
         <is>
-          <t>Logs, metrics, traces, alerts, dashboards</t>
+          <t>Reproducing bugs, hypothesis testing, debuggers, logging, bisecting</t>
         </is>
       </c>
     </row>
@@ -2702,46 +2684,46 @@
       <c r="B151" s="18" t="n"/>
       <c r="C151" s="18" t="inlineStr">
         <is>
-          <t>Incident Response and Postmortems</t>
+          <t>Writing Good Bug Reports</t>
         </is>
       </c>
       <c r="D151" s="18" t="inlineStr">
         <is>
-          <t>On-call, severity levels, blameless postmortems, learning culture</t>
+          <t>Steps to reproduce, expected vs actual, severity, triage</t>
         </is>
       </c>
     </row>
     <row r="152" s="16">
-      <c r="A152" s="18" t="n"/>
-      <c r="B152" s="18" t="n"/>
+      <c r="A152" s="18" t="n">
+        <v>11</v>
+      </c>
+      <c r="B152" s="18" t="inlineStr">
+        <is>
+          <t>Quality Assurance &amp; Verification</t>
+        </is>
+      </c>
       <c r="C152" s="18" t="inlineStr">
         <is>
-          <t>The DevOps Culture</t>
+          <t>Software Quality: Definitions and Models</t>
         </is>
       </c>
       <c r="D152" s="18" t="inlineStr">
         <is>
-          <t>Shared ownership, automation, measurement, DORA metrics</t>
+          <t>Quality attributes, ISO/IEC 25010, quality in use</t>
         </is>
       </c>
     </row>
     <row r="153" s="16">
-      <c r="A153" s="18" t="n">
-        <v>14</v>
-      </c>
-      <c r="B153" s="18" t="inlineStr">
-        <is>
-          <t>APIs, Data &amp; Persistence for Engineers</t>
-        </is>
-      </c>
+      <c r="A153" s="18" t="n"/>
+      <c r="B153" s="18" t="n"/>
       <c r="C153" s="18" t="inlineStr">
         <is>
-          <t>What Is an API?</t>
+          <t>Quality Assurance vs Quality Control</t>
         </is>
       </c>
       <c r="D153" s="18" t="inlineStr">
         <is>
-          <t>Contracts, libraries vs services, consumers and providers</t>
+          <t>Process focus vs product focus, QA activities</t>
         </is>
       </c>
     </row>
@@ -2750,12 +2732,12 @@
       <c r="B154" s="18" t="n"/>
       <c r="C154" s="18" t="inlineStr">
         <is>
-          <t>Designing REST APIs</t>
+          <t>Code Reviews and Inspections</t>
         </is>
       </c>
       <c r="D154" s="18" t="inlineStr">
         <is>
-          <t>Resources, HTTP verbs, status codes, statelessness</t>
+          <t>Walkthroughs, formal inspection, checklists, review etiquette</t>
         </is>
       </c>
     </row>
@@ -2764,12 +2746,12 @@
       <c r="B155" s="18" t="n"/>
       <c r="C155" s="18" t="inlineStr">
         <is>
-          <t>API Versioning, Documentation and Evolution</t>
+          <t>Static Analysis and Linting</t>
         </is>
       </c>
       <c r="D155" s="18" t="inlineStr">
         <is>
-          <t>OpenAPI, backward compatibility, deprecation</t>
+          <t>Automated checks, bug patterns, false positives</t>
         </is>
       </c>
     </row>
@@ -2778,12 +2760,12 @@
       <c r="B156" s="18" t="n"/>
       <c r="C156" s="18" t="inlineStr">
         <is>
-          <t>Data Formats and Serialization</t>
+          <t>Software Metrics</t>
         </is>
       </c>
       <c r="D156" s="18" t="inlineStr">
         <is>
-          <t>JSON, XML, protocol buffers, schemas</t>
+          <t>Lines of code, cyclomatic complexity, coupling metrics, defect density</t>
         </is>
       </c>
     </row>
@@ -2792,12 +2774,12 @@
       <c r="B157" s="18" t="n"/>
       <c r="C157" s="18" t="inlineStr">
         <is>
-          <t>Relational Databases and SQL for Developers</t>
+          <t>Defect Management and Root-Cause Analysis</t>
         </is>
       </c>
       <c r="D157" s="18" t="inlineStr">
         <is>
-          <t>Tables, keys, queries, joins, normalization</t>
+          <t>Defect lifecycle, classification, five whys, prevention</t>
         </is>
       </c>
     </row>
@@ -2806,12 +2788,12 @@
       <c r="B158" s="18" t="n"/>
       <c r="C158" s="18" t="inlineStr">
         <is>
-          <t>Transactions and Data Integrity</t>
+          <t>Reliability and Availability Basics</t>
         </is>
       </c>
       <c r="D158" s="18" t="inlineStr">
         <is>
-          <t>ACID, constraints, consistency, concurrency issues</t>
+          <t>MTBF, MTTR, failure rates, fault tolerance</t>
         </is>
       </c>
     </row>
@@ -2820,12 +2802,12 @@
       <c r="B159" s="18" t="n"/>
       <c r="C159" s="18" t="inlineStr">
         <is>
-          <t>NoSQL and Choosing a Data Store</t>
+          <t>Formal Specification and Verification: An Introduction</t>
         </is>
       </c>
       <c r="D159" s="18" t="inlineStr">
         <is>
-          <t>Document, key-value, graph stores, trade-offs</t>
+          <t>Invariants, assertions, model checking, when formal methods pay off</t>
         </is>
       </c>
     </row>
@@ -2834,12 +2816,12 @@
       <c r="B160" s="18" t="n"/>
       <c r="C160" s="18" t="inlineStr">
         <is>
-          <t>Object–Relational Mapping and Data Access Layers</t>
+          <t>Safety-Critical Software</t>
         </is>
       </c>
       <c r="D160" s="18" t="inlineStr">
         <is>
-          <t>ORM, repositories, impedance mismatch, N+1 queries</t>
+          <t>Hazard analysis, standards, certification, case studies</t>
         </is>
       </c>
     </row>
@@ -2848,46 +2830,46 @@
       <c r="B161" s="18" t="n"/>
       <c r="C161" s="18" t="inlineStr">
         <is>
-          <t>Caching Basics</t>
+          <t>Learning from Failures</t>
         </is>
       </c>
       <c r="D161" s="18" t="inlineStr">
         <is>
-          <t>Cache types, invalidation, consistency, cache-aside</t>
+          <t>Therac-25, Ariane 5, Knight Capital, post-mortem analysis</t>
         </is>
       </c>
     </row>
     <row r="162" s="16">
-      <c r="A162" s="18" t="n"/>
-      <c r="B162" s="18" t="n"/>
+      <c r="A162" s="18" t="n">
+        <v>12</v>
+      </c>
+      <c r="B162" s="18" t="inlineStr">
+        <is>
+          <t>APIs, Data &amp; Persistence for Engineers</t>
+        </is>
+      </c>
       <c r="C162" s="18" t="inlineStr">
         <is>
-          <t>Concurrency in Application Code</t>
+          <t>What Is an API?</t>
         </is>
       </c>
       <c r="D162" s="18" t="inlineStr">
         <is>
-          <t>Threads, async, race conditions, shared state at an applied level</t>
+          <t>Contracts, libraries vs services, consumers and providers</t>
         </is>
       </c>
     </row>
     <row r="163" s="16">
-      <c r="A163" s="18" t="n">
-        <v>15</v>
-      </c>
-      <c r="B163" s="18" t="inlineStr">
-        <is>
-          <t>Software Maintenance &amp; Evolution</t>
-        </is>
-      </c>
+      <c r="A163" s="18" t="n"/>
+      <c r="B163" s="18" t="n"/>
       <c r="C163" s="18" t="inlineStr">
         <is>
-          <t>Why Software Changes</t>
+          <t>Designing REST APIs</t>
         </is>
       </c>
       <c r="D163" s="18" t="inlineStr">
         <is>
-          <t>Lehman's laws, corrective, adaptive, perfective, preventive maintenance</t>
+          <t>Resources, HTTP verbs, status codes, statelessness</t>
         </is>
       </c>
     </row>
@@ -2896,12 +2878,12 @@
       <c r="B164" s="18" t="n"/>
       <c r="C164" s="18" t="inlineStr">
         <is>
-          <t>The Cost of Maintenance</t>
+          <t>API Versioning, Documentation and Evolution</t>
         </is>
       </c>
       <c r="D164" s="18" t="inlineStr">
         <is>
-          <t>Maintenance share of lifecycle cost, factors affecting maintainability</t>
+          <t>OpenAPI, backward compatibility, deprecation</t>
         </is>
       </c>
     </row>
@@ -2910,12 +2892,12 @@
       <c r="B165" s="18" t="n"/>
       <c r="C165" s="18" t="inlineStr">
         <is>
-          <t>Change Impact Analysis</t>
+          <t>Data Formats and Serialization</t>
         </is>
       </c>
       <c r="D165" s="18" t="inlineStr">
         <is>
-          <t>Dependencies, ripple effects, risk of change</t>
+          <t>JSON, XML, protocol buffers, schemas</t>
         </is>
       </c>
     </row>
@@ -2924,12 +2906,12 @@
       <c r="B166" s="18" t="n"/>
       <c r="C166" s="18" t="inlineStr">
         <is>
-          <t>Reverse Engineering and Program Comprehension</t>
+          <t>Relational Databases and SQL for Developers</t>
         </is>
       </c>
       <c r="D166" s="18" t="inlineStr">
         <is>
-          <t>Understanding unfamiliar systems, tools, documentation recovery</t>
+          <t>Tables, keys, queries, joins, normalization</t>
         </is>
       </c>
     </row>
@@ -2938,12 +2920,12 @@
       <c r="B167" s="18" t="n"/>
       <c r="C167" s="18" t="inlineStr">
         <is>
-          <t>Reengineering and Modernization</t>
+          <t>Transactions and Data Integrity</t>
         </is>
       </c>
       <c r="D167" s="18" t="inlineStr">
         <is>
-          <t>Rewrite vs refactor, strangler pattern, migration planning</t>
+          <t>ACID, constraints, consistency, concurrency issues</t>
         </is>
       </c>
     </row>
@@ -2952,12 +2934,12 @@
       <c r="B168" s="18" t="n"/>
       <c r="C168" s="18" t="inlineStr">
         <is>
-          <t>Software Reuse</t>
+          <t>NoSQL and Choosing a Data Store</t>
         </is>
       </c>
       <c r="D168" s="18" t="inlineStr">
         <is>
-          <t>Libraries, frameworks, components, reuse benefits and costs</t>
+          <t>Document, key-value, graph stores, trade-offs</t>
         </is>
       </c>
     </row>
@@ -2966,12 +2948,12 @@
       <c r="B169" s="18" t="n"/>
       <c r="C169" s="18" t="inlineStr">
         <is>
-          <t>Software Documentation</t>
+          <t>Object–Relational Mapping and Data Access Layers</t>
         </is>
       </c>
       <c r="D169" s="18" t="inlineStr">
         <is>
-          <t>README, API docs, runbooks, living documentation</t>
+          <t>ORM, repositories, impedance mismatch, N+1 queries</t>
         </is>
       </c>
     </row>
@@ -2980,12 +2962,12 @@
       <c r="B170" s="18" t="n"/>
       <c r="C170" s="18" t="inlineStr">
         <is>
-          <t>Configuration Management and Release Management</t>
+          <t>Caching Basics</t>
         </is>
       </c>
       <c r="D170" s="18" t="inlineStr">
         <is>
-          <t>Baselines, change control boards, release planning</t>
+          <t>Cache types, invalidation, consistency, cache-aside</t>
         </is>
       </c>
     </row>
@@ -2994,18 +2976,18 @@
       <c r="B171" s="18" t="n"/>
       <c r="C171" s="18" t="inlineStr">
         <is>
-          <t>End of Life and Software Sustainability</t>
+          <t>Concurrency in Application Code</t>
         </is>
       </c>
       <c r="D171" s="18" t="inlineStr">
         <is>
-          <t>Deprecation, sunsetting, long-term support, green software</t>
+          <t>Threads, async, race conditions, shared state at an applied level</t>
         </is>
       </c>
     </row>
     <row r="172" s="16">
       <c r="A172" s="18" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B172" s="18" t="inlineStr">
         <is>
@@ -3151,11 +3133,11 @@
     </row>
     <row r="182" s="16">
       <c r="A182" s="18" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B182" s="18" t="inlineStr">
         <is>
-          <t>Secure Software Development</t>
+          <t>Security, Ethics &amp; Professional Practice</t>
         </is>
       </c>
       <c r="C182" s="18" t="inlineStr">
@@ -3282,14 +3264,8 @@
       </c>
     </row>
     <row r="191" s="16">
-      <c r="A191" s="18" t="n">
-        <v>18</v>
-      </c>
-      <c r="B191" s="18" t="inlineStr">
-        <is>
-          <t>Professional Practice, Ethics &amp; Modern Engineering</t>
-        </is>
-      </c>
+      <c r="A191" s="18" t="n"/>
+      <c r="B191" s="18" t="n"/>
       <c r="C191" s="18" t="inlineStr">
         <is>
           <t>Professional Ethics in Software Engineering</t>
@@ -4241,43 +4217,35 @@
     <row r="999" ht="15.75" customHeight="1" s="16"/>
     <row r="1000" ht="15.75" customHeight="1" s="16"/>
   </sheetData>
-  <mergeCells count="36">
+  <mergeCells count="28">
     <mergeCell ref="A2:A13"/>
-    <mergeCell ref="B182:B190"/>
-    <mergeCell ref="B191:B201"/>
-    <mergeCell ref="B117:B131"/>
+    <mergeCell ref="A152:A161"/>
+    <mergeCell ref="B182:B201"/>
+    <mergeCell ref="B114:B136"/>
+    <mergeCell ref="A137:A151"/>
     <mergeCell ref="A35:A46"/>
-    <mergeCell ref="A163:A171"/>
     <mergeCell ref="B35:B46"/>
     <mergeCell ref="A58:A69"/>
-    <mergeCell ref="B153:B162"/>
     <mergeCell ref="A172:A181"/>
-    <mergeCell ref="A132:A141"/>
-    <mergeCell ref="B142:B152"/>
-    <mergeCell ref="B24:B34"/>
+    <mergeCell ref="A114:A136"/>
     <mergeCell ref="B2:B13"/>
-    <mergeCell ref="B105:B116"/>
-    <mergeCell ref="A153:A162"/>
+    <mergeCell ref="B14:B34"/>
+    <mergeCell ref="A162:A171"/>
     <mergeCell ref="A70:A81"/>
     <mergeCell ref="A82:A93"/>
+    <mergeCell ref="B152:B161"/>
     <mergeCell ref="A47:A57"/>
-    <mergeCell ref="B14:B23"/>
+    <mergeCell ref="B137:B151"/>
+    <mergeCell ref="B94:B113"/>
     <mergeCell ref="B58:B69"/>
-    <mergeCell ref="A182:A190"/>
     <mergeCell ref="B70:B81"/>
-    <mergeCell ref="B132:B141"/>
-    <mergeCell ref="A24:A34"/>
-    <mergeCell ref="A142:A152"/>
-    <mergeCell ref="B163:B171"/>
     <mergeCell ref="B172:B181"/>
-    <mergeCell ref="A105:A116"/>
+    <mergeCell ref="A14:A34"/>
+    <mergeCell ref="B162:B171"/>
     <mergeCell ref="B82:B93"/>
-    <mergeCell ref="B94:B104"/>
+    <mergeCell ref="A182:A201"/>
     <mergeCell ref="B47:B57"/>
-    <mergeCell ref="A14:A23"/>
-    <mergeCell ref="A117:A131"/>
-    <mergeCell ref="A191:A201"/>
-    <mergeCell ref="A94:A104"/>
+    <mergeCell ref="A94:A113"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -4594,7 +4562,7 @@
       </c>
       <c r="B14" s="19" t="inlineStr">
         <is>
-          <t>software-process-models</t>
+          <t>software-process-models-and-agile-methods</t>
         </is>
       </c>
       <c r="C14" s="19" t="inlineStr">
@@ -4616,7 +4584,7 @@
       </c>
       <c r="B15" s="19" t="inlineStr">
         <is>
-          <t>software-process-models</t>
+          <t>software-process-models-and-agile-methods</t>
         </is>
       </c>
       <c r="C15" s="19" t="inlineStr">
@@ -4638,7 +4606,7 @@
       </c>
       <c r="B16" s="19" t="inlineStr">
         <is>
-          <t>software-process-models</t>
+          <t>software-process-models-and-agile-methods</t>
         </is>
       </c>
       <c r="C16" s="19" t="inlineStr">
@@ -4660,7 +4628,7 @@
       </c>
       <c r="B17" s="19" t="inlineStr">
         <is>
-          <t>software-process-models</t>
+          <t>software-process-models-and-agile-methods</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
@@ -4682,7 +4650,7 @@
       </c>
       <c r="B18" s="19" t="inlineStr">
         <is>
-          <t>software-process-models</t>
+          <t>software-process-models-and-agile-methods</t>
         </is>
       </c>
       <c r="C18" s="19" t="inlineStr">
@@ -4704,7 +4672,7 @@
       </c>
       <c r="B19" s="19" t="inlineStr">
         <is>
-          <t>software-process-models</t>
+          <t>software-process-models-and-agile-methods</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
@@ -4726,7 +4694,7 @@
       </c>
       <c r="B20" s="19" t="inlineStr">
         <is>
-          <t>software-process-models</t>
+          <t>software-process-models-and-agile-methods</t>
         </is>
       </c>
       <c r="C20" s="19" t="inlineStr">
@@ -4748,7 +4716,7 @@
       </c>
       <c r="B21" s="19" t="inlineStr">
         <is>
-          <t>software-process-models</t>
+          <t>software-process-models-and-agile-methods</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
@@ -4770,7 +4738,7 @@
       </c>
       <c r="B22" s="19" t="inlineStr">
         <is>
-          <t>software-process-models</t>
+          <t>software-process-models-and-agile-methods</t>
         </is>
       </c>
       <c r="C22" s="19" t="inlineStr">
@@ -4792,7 +4760,7 @@
       </c>
       <c r="B23" s="19" t="inlineStr">
         <is>
-          <t>software-process-models</t>
+          <t>software-process-models-and-agile-methods</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
@@ -4814,7 +4782,7 @@
       </c>
       <c r="B24" s="19" t="inlineStr">
         <is>
-          <t>agile-methods-and-team-practices</t>
+          <t>software-process-models-and-agile-methods</t>
         </is>
       </c>
       <c r="C24" s="19" t="inlineStr">
@@ -4836,7 +4804,7 @@
       </c>
       <c r="B25" s="19" t="inlineStr">
         <is>
-          <t>agile-methods-and-team-practices</t>
+          <t>software-process-models-and-agile-methods</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
@@ -4858,7 +4826,7 @@
       </c>
       <c r="B26" s="19" t="inlineStr">
         <is>
-          <t>agile-methods-and-team-practices</t>
+          <t>software-process-models-and-agile-methods</t>
         </is>
       </c>
       <c r="C26" s="19" t="inlineStr">
@@ -4880,7 +4848,7 @@
       </c>
       <c r="B27" s="19" t="inlineStr">
         <is>
-          <t>agile-methods-and-team-practices</t>
+          <t>software-process-models-and-agile-methods</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
@@ -4902,7 +4870,7 @@
       </c>
       <c r="B28" s="19" t="inlineStr">
         <is>
-          <t>agile-methods-and-team-practices</t>
+          <t>software-process-models-and-agile-methods</t>
         </is>
       </c>
       <c r="C28" s="19" t="inlineStr">
@@ -4924,7 +4892,7 @@
       </c>
       <c r="B29" s="19" t="inlineStr">
         <is>
-          <t>agile-methods-and-team-practices</t>
+          <t>software-process-models-and-agile-methods</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
@@ -4946,7 +4914,7 @@
       </c>
       <c r="B30" s="19" t="inlineStr">
         <is>
-          <t>agile-methods-and-team-practices</t>
+          <t>software-process-models-and-agile-methods</t>
         </is>
       </c>
       <c r="C30" s="19" t="inlineStr">
@@ -4968,7 +4936,7 @@
       </c>
       <c r="B31" s="19" t="inlineStr">
         <is>
-          <t>agile-methods-and-team-practices</t>
+          <t>software-process-models-and-agile-methods</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
@@ -4990,7 +4958,7 @@
       </c>
       <c r="B32" s="19" t="inlineStr">
         <is>
-          <t>agile-methods-and-team-practices</t>
+          <t>software-process-models-and-agile-methods</t>
         </is>
       </c>
       <c r="C32" s="19" t="inlineStr">
@@ -5012,7 +4980,7 @@
       </c>
       <c r="B33" s="19" t="inlineStr">
         <is>
-          <t>agile-methods-and-team-practices</t>
+          <t>software-process-models-and-agile-methods</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
@@ -5034,7 +5002,7 @@
       </c>
       <c r="B34" s="19" t="inlineStr">
         <is>
-          <t>agile-methods-and-team-practices</t>
+          <t>software-process-models-and-agile-methods</t>
         </is>
       </c>
       <c r="C34" s="19" t="inlineStr">
@@ -6354,7 +6322,7 @@
       </c>
       <c r="B94" s="19" t="inlineStr">
         <is>
-          <t>clean-code-and-refactoring</t>
+          <t>clean-code-refactoring-and-software-evolution</t>
         </is>
       </c>
       <c r="C94" s="19" t="inlineStr">
@@ -6376,7 +6344,7 @@
       </c>
       <c r="B95" s="19" t="inlineStr">
         <is>
-          <t>clean-code-and-refactoring</t>
+          <t>clean-code-refactoring-and-software-evolution</t>
         </is>
       </c>
       <c r="C95" s="19" t="inlineStr">
@@ -6398,7 +6366,7 @@
       </c>
       <c r="B96" s="19" t="inlineStr">
         <is>
-          <t>clean-code-and-refactoring</t>
+          <t>clean-code-refactoring-and-software-evolution</t>
         </is>
       </c>
       <c r="C96" s="19" t="inlineStr">
@@ -6420,7 +6388,7 @@
       </c>
       <c r="B97" s="19" t="inlineStr">
         <is>
-          <t>clean-code-and-refactoring</t>
+          <t>clean-code-refactoring-and-software-evolution</t>
         </is>
       </c>
       <c r="C97" s="19" t="inlineStr">
@@ -6442,7 +6410,7 @@
       </c>
       <c r="B98" s="19" t="inlineStr">
         <is>
-          <t>clean-code-and-refactoring</t>
+          <t>clean-code-refactoring-and-software-evolution</t>
         </is>
       </c>
       <c r="C98" s="19" t="inlineStr">
@@ -6464,7 +6432,7 @@
       </c>
       <c r="B99" s="19" t="inlineStr">
         <is>
-          <t>clean-code-and-refactoring</t>
+          <t>clean-code-refactoring-and-software-evolution</t>
         </is>
       </c>
       <c r="C99" s="19" t="inlineStr">
@@ -6486,7 +6454,7 @@
       </c>
       <c r="B100" s="19" t="inlineStr">
         <is>
-          <t>clean-code-and-refactoring</t>
+          <t>clean-code-refactoring-and-software-evolution</t>
         </is>
       </c>
       <c r="C100" s="19" t="inlineStr">
@@ -6508,7 +6476,7 @@
       </c>
       <c r="B101" s="19" t="inlineStr">
         <is>
-          <t>clean-code-and-refactoring</t>
+          <t>clean-code-refactoring-and-software-evolution</t>
         </is>
       </c>
       <c r="C101" s="19" t="inlineStr">
@@ -6530,7 +6498,7 @@
       </c>
       <c r="B102" s="19" t="inlineStr">
         <is>
-          <t>clean-code-and-refactoring</t>
+          <t>clean-code-refactoring-and-software-evolution</t>
         </is>
       </c>
       <c r="C102" s="19" t="inlineStr">
@@ -6552,7 +6520,7 @@
       </c>
       <c r="B103" s="19" t="inlineStr">
         <is>
-          <t>clean-code-and-refactoring</t>
+          <t>clean-code-refactoring-and-software-evolution</t>
         </is>
       </c>
       <c r="C103" s="19" t="inlineStr">
@@ -6574,7 +6542,7 @@
       </c>
       <c r="B104" s="19" t="inlineStr">
         <is>
-          <t>clean-code-and-refactoring</t>
+          <t>clean-code-refactoring-and-software-evolution</t>
         </is>
       </c>
       <c r="C104" s="19" t="inlineStr">
@@ -6596,12 +6564,12 @@
       </c>
       <c r="B105" s="19" t="inlineStr">
         <is>
-          <t>version-control-and-collaboration</t>
+          <t>clean-code-refactoring-and-software-evolution</t>
         </is>
       </c>
       <c r="C105" s="19" t="inlineStr">
         <is>
-          <t>why-version-control</t>
+          <t>why-software-changes</t>
         </is>
       </c>
       <c r="D105" s="19" t="inlineStr">
@@ -6618,12 +6586,12 @@
       </c>
       <c r="B106" s="19" t="inlineStr">
         <is>
-          <t>version-control-and-collaboration</t>
+          <t>clean-code-refactoring-and-software-evolution</t>
         </is>
       </c>
       <c r="C106" s="19" t="inlineStr">
         <is>
-          <t>git-fundamentals</t>
+          <t>the-cost-of-maintenance</t>
         </is>
       </c>
       <c r="D106" s="19" t="inlineStr">
@@ -6640,12 +6608,12 @@
       </c>
       <c r="B107" s="19" t="inlineStr">
         <is>
-          <t>version-control-and-collaboration</t>
+          <t>clean-code-refactoring-and-software-evolution</t>
         </is>
       </c>
       <c r="C107" s="19" t="inlineStr">
         <is>
-          <t>commits-history-and-good-commit-messages</t>
+          <t>change-impact-analysis</t>
         </is>
       </c>
       <c r="D107" s="19" t="inlineStr">
@@ -6662,12 +6630,12 @@
       </c>
       <c r="B108" s="19" t="inlineStr">
         <is>
-          <t>version-control-and-collaboration</t>
+          <t>clean-code-refactoring-and-software-evolution</t>
         </is>
       </c>
       <c r="C108" s="19" t="inlineStr">
         <is>
-          <t>branching-and-merging</t>
+          <t>reverse-engineering-and-program-comprehension</t>
         </is>
       </c>
       <c r="D108" s="19" t="inlineStr">
@@ -6684,12 +6652,12 @@
       </c>
       <c r="B109" s="19" t="inlineStr">
         <is>
-          <t>version-control-and-collaboration</t>
+          <t>clean-code-refactoring-and-software-evolution</t>
         </is>
       </c>
       <c r="C109" s="19" t="inlineStr">
         <is>
-          <t>resolving-merge-conflicts</t>
+          <t>reengineering-and-modernization</t>
         </is>
       </c>
       <c r="D109" s="19" t="inlineStr">
@@ -6706,12 +6674,12 @@
       </c>
       <c r="B110" s="19" t="inlineStr">
         <is>
-          <t>version-control-and-collaboration</t>
+          <t>clean-code-refactoring-and-software-evolution</t>
         </is>
       </c>
       <c r="C110" s="19" t="inlineStr">
         <is>
-          <t>remote-repositories-and-collaboration</t>
+          <t>software-reuse</t>
         </is>
       </c>
       <c r="D110" s="19" t="inlineStr">
@@ -6728,12 +6696,12 @@
       </c>
       <c r="B111" s="19" t="inlineStr">
         <is>
-          <t>version-control-and-collaboration</t>
+          <t>clean-code-refactoring-and-software-evolution</t>
         </is>
       </c>
       <c r="C111" s="19" t="inlineStr">
         <is>
-          <t>branching-strategies</t>
+          <t>software-documentation</t>
         </is>
       </c>
       <c r="D111" s="19" t="inlineStr">
@@ -6750,12 +6718,12 @@
       </c>
       <c r="B112" s="19" t="inlineStr">
         <is>
-          <t>version-control-and-collaboration</t>
+          <t>clean-code-refactoring-and-software-evolution</t>
         </is>
       </c>
       <c r="C112" s="19" t="inlineStr">
         <is>
-          <t>pull-requests-and-code-review-workflow</t>
+          <t>configuration-management-and-release-management</t>
         </is>
       </c>
       <c r="D112" s="19" t="inlineStr">
@@ -6772,12 +6740,12 @@
       </c>
       <c r="B113" s="19" t="inlineStr">
         <is>
-          <t>version-control-and-collaboration</t>
+          <t>clean-code-refactoring-and-software-evolution</t>
         </is>
       </c>
       <c r="C113" s="19" t="inlineStr">
         <is>
-          <t>rebasing-cherry-picking-and-rewriting-history</t>
+          <t>end-of-life-and-software-sustainability</t>
         </is>
       </c>
       <c r="D113" s="19" t="inlineStr">
@@ -6794,12 +6762,12 @@
       </c>
       <c r="B114" s="19" t="inlineStr">
         <is>
-          <t>version-control-and-collaboration</t>
+          <t>version-control-build-and-devops</t>
         </is>
       </c>
       <c r="C114" s="19" t="inlineStr">
         <is>
-          <t>tags-releases-and-semantic-versioning</t>
+          <t>why-version-control</t>
         </is>
       </c>
       <c r="D114" s="19" t="inlineStr">
@@ -6816,12 +6784,12 @@
       </c>
       <c r="B115" s="19" t="inlineStr">
         <is>
-          <t>version-control-and-collaboration</t>
+          <t>version-control-build-and-devops</t>
         </is>
       </c>
       <c r="C115" s="19" t="inlineStr">
         <is>
-          <t>issue-tracking-and-project-boards</t>
+          <t>git-fundamentals</t>
         </is>
       </c>
       <c r="D115" s="19" t="inlineStr">
@@ -6838,12 +6806,12 @@
       </c>
       <c r="B116" s="19" t="inlineStr">
         <is>
-          <t>version-control-and-collaboration</t>
+          <t>version-control-build-and-devops</t>
         </is>
       </c>
       <c r="C116" s="19" t="inlineStr">
         <is>
-          <t>open-source-collaboration</t>
+          <t>commits-history-and-good-commit-messages</t>
         </is>
       </c>
       <c r="D116" s="19" t="inlineStr">
@@ -6860,12 +6828,12 @@
       </c>
       <c r="B117" s="19" t="inlineStr">
         <is>
-          <t>software-testing-fundamentals</t>
+          <t>version-control-build-and-devops</t>
         </is>
       </c>
       <c r="C117" s="19" t="inlineStr">
         <is>
-          <t>why-test-software</t>
+          <t>branching-and-merging</t>
         </is>
       </c>
       <c r="D117" s="19" t="inlineStr">
@@ -6882,12 +6850,12 @@
       </c>
       <c r="B118" s="19" t="inlineStr">
         <is>
-          <t>software-testing-fundamentals</t>
+          <t>version-control-build-and-devops</t>
         </is>
       </c>
       <c r="C118" s="19" t="inlineStr">
         <is>
-          <t>testing-terminology-and-the-test-pyramid</t>
+          <t>resolving-merge-conflicts</t>
         </is>
       </c>
       <c r="D118" s="19" t="inlineStr">
@@ -6904,12 +6872,12 @@
       </c>
       <c r="B119" s="19" t="inlineStr">
         <is>
-          <t>software-testing-fundamentals</t>
+          <t>version-control-build-and-devops</t>
         </is>
       </c>
       <c r="C119" s="19" t="inlineStr">
         <is>
-          <t>unit-testing</t>
+          <t>remote-repositories-and-collaboration</t>
         </is>
       </c>
       <c r="D119" s="19" t="inlineStr">
@@ -6926,12 +6894,12 @@
       </c>
       <c r="B120" s="19" t="inlineStr">
         <is>
-          <t>software-testing-fundamentals</t>
+          <t>version-control-build-and-devops</t>
         </is>
       </c>
       <c r="C120" s="19" t="inlineStr">
         <is>
-          <t>test-design-equivalence-partitioning-and-boundary-value-analysis</t>
+          <t>branching-strategies</t>
         </is>
       </c>
       <c r="D120" s="19" t="inlineStr">
@@ -6948,12 +6916,12 @@
       </c>
       <c r="B121" s="19" t="inlineStr">
         <is>
-          <t>software-testing-fundamentals</t>
+          <t>version-control-build-and-devops</t>
         </is>
       </c>
       <c r="C121" s="19" t="inlineStr">
         <is>
-          <t>test-design-decision-tables-and-state-based-testing</t>
+          <t>pull-requests-and-code-review-workflow</t>
         </is>
       </c>
       <c r="D121" s="19" t="inlineStr">
@@ -6970,12 +6938,12 @@
       </c>
       <c r="B122" s="19" t="inlineStr">
         <is>
-          <t>software-testing-fundamentals</t>
+          <t>version-control-build-and-devops</t>
         </is>
       </c>
       <c r="C122" s="19" t="inlineStr">
         <is>
-          <t>white-box-testing-and-code-coverage</t>
+          <t>rebasing-cherry-picking-and-rewriting-history</t>
         </is>
       </c>
       <c r="D122" s="19" t="inlineStr">
@@ -6992,12 +6960,12 @@
       </c>
       <c r="B123" s="19" t="inlineStr">
         <is>
-          <t>software-testing-fundamentals</t>
+          <t>version-control-build-and-devops</t>
         </is>
       </c>
       <c r="C123" s="19" t="inlineStr">
         <is>
-          <t>test-doubles-stubs-mocks-and-fakes</t>
+          <t>tags-releases-and-semantic-versioning</t>
         </is>
       </c>
       <c r="D123" s="19" t="inlineStr">
@@ -7014,12 +6982,12 @@
       </c>
       <c r="B124" s="19" t="inlineStr">
         <is>
-          <t>software-testing-fundamentals</t>
+          <t>version-control-build-and-devops</t>
         </is>
       </c>
       <c r="C124" s="19" t="inlineStr">
         <is>
-          <t>test-driven-development</t>
+          <t>issue-tracking-and-project-boards</t>
         </is>
       </c>
       <c r="D124" s="19" t="inlineStr">
@@ -7036,12 +7004,12 @@
       </c>
       <c r="B125" s="19" t="inlineStr">
         <is>
-          <t>software-testing-fundamentals</t>
+          <t>version-control-build-and-devops</t>
         </is>
       </c>
       <c r="C125" s="19" t="inlineStr">
         <is>
-          <t>behaviour-driven-development</t>
+          <t>open-source-collaboration</t>
         </is>
       </c>
       <c r="D125" s="19" t="inlineStr">
@@ -7058,12 +7026,12 @@
       </c>
       <c r="B126" s="19" t="inlineStr">
         <is>
-          <t>software-testing-fundamentals</t>
+          <t>version-control-build-and-devops</t>
         </is>
       </c>
       <c r="C126" s="19" t="inlineStr">
         <is>
-          <t>integration-and-system-testing</t>
+          <t>from-source-code-to-deployable-software</t>
         </is>
       </c>
       <c r="D126" s="19" t="inlineStr">
@@ -7080,12 +7048,12 @@
       </c>
       <c r="B127" s="19" t="inlineStr">
         <is>
-          <t>software-testing-fundamentals</t>
+          <t>version-control-build-and-devops</t>
         </is>
       </c>
       <c r="C127" s="19" t="inlineStr">
         <is>
-          <t>regression-testing-and-test-automation</t>
+          <t>build-tools-and-dependency-management</t>
         </is>
       </c>
       <c r="D127" s="19" t="inlineStr">
@@ -7102,12 +7070,12 @@
       </c>
       <c r="B128" s="19" t="inlineStr">
         <is>
-          <t>software-testing-fundamentals</t>
+          <t>version-control-build-and-devops</t>
         </is>
       </c>
       <c r="C128" s="19" t="inlineStr">
         <is>
-          <t>acceptance-exploratory-and-usability-testing</t>
+          <t>continuous-integration</t>
         </is>
       </c>
       <c r="D128" s="19" t="inlineStr">
@@ -7124,12 +7092,12 @@
       </c>
       <c r="B129" s="19" t="inlineStr">
         <is>
-          <t>software-testing-fundamentals</t>
+          <t>version-control-build-and-devops</t>
         </is>
       </c>
       <c r="C129" s="19" t="inlineStr">
         <is>
-          <t>non-functional-testing</t>
+          <t>continuous-delivery-and-deployment</t>
         </is>
       </c>
       <c r="D129" s="19" t="inlineStr">
@@ -7146,12 +7114,12 @@
       </c>
       <c r="B130" s="19" t="inlineStr">
         <is>
-          <t>software-testing-fundamentals</t>
+          <t>version-control-build-and-devops</t>
         </is>
       </c>
       <c r="C130" s="19" t="inlineStr">
         <is>
-          <t>debugging-systematically</t>
+          <t>environments-and-configuration-management</t>
         </is>
       </c>
       <c r="D130" s="19" t="inlineStr">
@@ -7168,12 +7136,12 @@
       </c>
       <c r="B131" s="19" t="inlineStr">
         <is>
-          <t>software-testing-fundamentals</t>
+          <t>version-control-build-and-devops</t>
         </is>
       </c>
       <c r="C131" s="19" t="inlineStr">
         <is>
-          <t>writing-good-bug-reports</t>
+          <t>containers-for-developers</t>
         </is>
       </c>
       <c r="D131" s="19" t="inlineStr">
@@ -7190,12 +7158,12 @@
       </c>
       <c r="B132" s="19" t="inlineStr">
         <is>
-          <t>quality-assurance-and-verification</t>
+          <t>version-control-build-and-devops</t>
         </is>
       </c>
       <c r="C132" s="19" t="inlineStr">
         <is>
-          <t>software-quality-definitions-and-models</t>
+          <t>infrastructure-as-code</t>
         </is>
       </c>
       <c r="D132" s="19" t="inlineStr">
@@ -7212,12 +7180,12 @@
       </c>
       <c r="B133" s="19" t="inlineStr">
         <is>
-          <t>quality-assurance-and-verification</t>
+          <t>version-control-build-and-devops</t>
         </is>
       </c>
       <c r="C133" s="19" t="inlineStr">
         <is>
-          <t>quality-assurance-vs-quality-control</t>
+          <t>release-strategies</t>
         </is>
       </c>
       <c r="D133" s="19" t="inlineStr">
@@ -7234,12 +7202,12 @@
       </c>
       <c r="B134" s="19" t="inlineStr">
         <is>
-          <t>quality-assurance-and-verification</t>
+          <t>version-control-build-and-devops</t>
         </is>
       </c>
       <c r="C134" s="19" t="inlineStr">
         <is>
-          <t>code-reviews-and-inspections</t>
+          <t>monitoring-logging-and-observability</t>
         </is>
       </c>
       <c r="D134" s="19" t="inlineStr">
@@ -7256,12 +7224,12 @@
       </c>
       <c r="B135" s="19" t="inlineStr">
         <is>
-          <t>quality-assurance-and-verification</t>
+          <t>version-control-build-and-devops</t>
         </is>
       </c>
       <c r="C135" s="19" t="inlineStr">
         <is>
-          <t>static-analysis-and-linting</t>
+          <t>incident-response-and-postmortems</t>
         </is>
       </c>
       <c r="D135" s="19" t="inlineStr">
@@ -7278,12 +7246,12 @@
       </c>
       <c r="B136" s="19" t="inlineStr">
         <is>
-          <t>quality-assurance-and-verification</t>
+          <t>version-control-build-and-devops</t>
         </is>
       </c>
       <c r="C136" s="19" t="inlineStr">
         <is>
-          <t>software-metrics</t>
+          <t>the-devops-culture</t>
         </is>
       </c>
       <c r="D136" s="19" t="inlineStr">
@@ -7300,12 +7268,12 @@
       </c>
       <c r="B137" s="19" t="inlineStr">
         <is>
-          <t>quality-assurance-and-verification</t>
+          <t>software-testing-fundamentals</t>
         </is>
       </c>
       <c r="C137" s="19" t="inlineStr">
         <is>
-          <t>defect-management-and-root-cause-analysis</t>
+          <t>why-test-software</t>
         </is>
       </c>
       <c r="D137" s="19" t="inlineStr">
@@ -7322,12 +7290,12 @@
       </c>
       <c r="B138" s="19" t="inlineStr">
         <is>
-          <t>quality-assurance-and-verification</t>
+          <t>software-testing-fundamentals</t>
         </is>
       </c>
       <c r="C138" s="19" t="inlineStr">
         <is>
-          <t>reliability-and-availability-basics</t>
+          <t>testing-terminology-and-the-test-pyramid</t>
         </is>
       </c>
       <c r="D138" s="19" t="inlineStr">
@@ -7344,12 +7312,12 @@
       </c>
       <c r="B139" s="19" t="inlineStr">
         <is>
-          <t>quality-assurance-and-verification</t>
+          <t>software-testing-fundamentals</t>
         </is>
       </c>
       <c r="C139" s="19" t="inlineStr">
         <is>
-          <t>formal-specification-and-verification-an-introduction</t>
+          <t>unit-testing</t>
         </is>
       </c>
       <c r="D139" s="19" t="inlineStr">
@@ -7366,12 +7334,12 @@
       </c>
       <c r="B140" s="19" t="inlineStr">
         <is>
-          <t>quality-assurance-and-verification</t>
+          <t>software-testing-fundamentals</t>
         </is>
       </c>
       <c r="C140" s="19" t="inlineStr">
         <is>
-          <t>safety-critical-software</t>
+          <t>test-design-equivalence-partitioning-and-boundary-value-analysis</t>
         </is>
       </c>
       <c r="D140" s="19" t="inlineStr">
@@ -7388,12 +7356,12 @@
       </c>
       <c r="B141" s="19" t="inlineStr">
         <is>
-          <t>quality-assurance-and-verification</t>
+          <t>software-testing-fundamentals</t>
         </is>
       </c>
       <c r="C141" s="19" t="inlineStr">
         <is>
-          <t>learning-from-failures</t>
+          <t>test-design-decision-tables-and-state-based-testing</t>
         </is>
       </c>
       <c r="D141" s="19" t="inlineStr">
@@ -7410,12 +7378,12 @@
       </c>
       <c r="B142" s="19" t="inlineStr">
         <is>
-          <t>build-release-and-devops</t>
+          <t>software-testing-fundamentals</t>
         </is>
       </c>
       <c r="C142" s="19" t="inlineStr">
         <is>
-          <t>from-source-code-to-deployable-software</t>
+          <t>white-box-testing-and-code-coverage</t>
         </is>
       </c>
       <c r="D142" s="19" t="inlineStr">
@@ -7432,12 +7400,12 @@
       </c>
       <c r="B143" s="19" t="inlineStr">
         <is>
-          <t>build-release-and-devops</t>
+          <t>software-testing-fundamentals</t>
         </is>
       </c>
       <c r="C143" s="19" t="inlineStr">
         <is>
-          <t>build-tools-and-dependency-management</t>
+          <t>test-doubles-stubs-mocks-and-fakes</t>
         </is>
       </c>
       <c r="D143" s="19" t="inlineStr">
@@ -7454,12 +7422,12 @@
       </c>
       <c r="B144" s="19" t="inlineStr">
         <is>
-          <t>build-release-and-devops</t>
+          <t>software-testing-fundamentals</t>
         </is>
       </c>
       <c r="C144" s="19" t="inlineStr">
         <is>
-          <t>continuous-integration</t>
+          <t>test-driven-development</t>
         </is>
       </c>
       <c r="D144" s="19" t="inlineStr">
@@ -7476,12 +7444,12 @@
       </c>
       <c r="B145" s="19" t="inlineStr">
         <is>
-          <t>build-release-and-devops</t>
+          <t>software-testing-fundamentals</t>
         </is>
       </c>
       <c r="C145" s="19" t="inlineStr">
         <is>
-          <t>continuous-delivery-and-deployment</t>
+          <t>behaviour-driven-development</t>
         </is>
       </c>
       <c r="D145" s="19" t="inlineStr">
@@ -7498,12 +7466,12 @@
       </c>
       <c r="B146" s="19" t="inlineStr">
         <is>
-          <t>build-release-and-devops</t>
+          <t>software-testing-fundamentals</t>
         </is>
       </c>
       <c r="C146" s="19" t="inlineStr">
         <is>
-          <t>environments-and-configuration-management</t>
+          <t>integration-and-system-testing</t>
         </is>
       </c>
       <c r="D146" s="19" t="inlineStr">
@@ -7520,12 +7488,12 @@
       </c>
       <c r="B147" s="19" t="inlineStr">
         <is>
-          <t>build-release-and-devops</t>
+          <t>software-testing-fundamentals</t>
         </is>
       </c>
       <c r="C147" s="19" t="inlineStr">
         <is>
-          <t>containers-for-developers</t>
+          <t>regression-testing-and-test-automation</t>
         </is>
       </c>
       <c r="D147" s="19" t="inlineStr">
@@ -7542,12 +7510,12 @@
       </c>
       <c r="B148" s="19" t="inlineStr">
         <is>
-          <t>build-release-and-devops</t>
+          <t>software-testing-fundamentals</t>
         </is>
       </c>
       <c r="C148" s="19" t="inlineStr">
         <is>
-          <t>infrastructure-as-code</t>
+          <t>acceptance-exploratory-and-usability-testing</t>
         </is>
       </c>
       <c r="D148" s="19" t="inlineStr">
@@ -7564,12 +7532,12 @@
       </c>
       <c r="B149" s="19" t="inlineStr">
         <is>
-          <t>build-release-and-devops</t>
+          <t>software-testing-fundamentals</t>
         </is>
       </c>
       <c r="C149" s="19" t="inlineStr">
         <is>
-          <t>release-strategies</t>
+          <t>non-functional-testing</t>
         </is>
       </c>
       <c r="D149" s="19" t="inlineStr">
@@ -7586,12 +7554,12 @@
       </c>
       <c r="B150" s="19" t="inlineStr">
         <is>
-          <t>build-release-and-devops</t>
+          <t>software-testing-fundamentals</t>
         </is>
       </c>
       <c r="C150" s="19" t="inlineStr">
         <is>
-          <t>monitoring-logging-and-observability</t>
+          <t>debugging-systematically</t>
         </is>
       </c>
       <c r="D150" s="19" t="inlineStr">
@@ -7608,12 +7576,12 @@
       </c>
       <c r="B151" s="19" t="inlineStr">
         <is>
-          <t>build-release-and-devops</t>
+          <t>software-testing-fundamentals</t>
         </is>
       </c>
       <c r="C151" s="19" t="inlineStr">
         <is>
-          <t>incident-response-and-postmortems</t>
+          <t>writing-good-bug-reports</t>
         </is>
       </c>
       <c r="D151" s="19" t="inlineStr">
@@ -7630,12 +7598,12 @@
       </c>
       <c r="B152" s="19" t="inlineStr">
         <is>
-          <t>build-release-and-devops</t>
+          <t>quality-assurance-and-verification</t>
         </is>
       </c>
       <c r="C152" s="19" t="inlineStr">
         <is>
-          <t>the-devops-culture</t>
+          <t>software-quality-definitions-and-models</t>
         </is>
       </c>
       <c r="D152" s="19" t="inlineStr">
@@ -7652,12 +7620,12 @@
       </c>
       <c r="B153" s="19" t="inlineStr">
         <is>
-          <t>apis-data-and-persistence-for-engineers</t>
+          <t>quality-assurance-and-verification</t>
         </is>
       </c>
       <c r="C153" s="19" t="inlineStr">
         <is>
-          <t>what-is-an-api</t>
+          <t>quality-assurance-vs-quality-control</t>
         </is>
       </c>
       <c r="D153" s="19" t="inlineStr">
@@ -7674,12 +7642,12 @@
       </c>
       <c r="B154" s="19" t="inlineStr">
         <is>
-          <t>apis-data-and-persistence-for-engineers</t>
+          <t>quality-assurance-and-verification</t>
         </is>
       </c>
       <c r="C154" s="19" t="inlineStr">
         <is>
-          <t>designing-rest-apis</t>
+          <t>code-reviews-and-inspections</t>
         </is>
       </c>
       <c r="D154" s="19" t="inlineStr">
@@ -7696,12 +7664,12 @@
       </c>
       <c r="B155" s="19" t="inlineStr">
         <is>
-          <t>apis-data-and-persistence-for-engineers</t>
+          <t>quality-assurance-and-verification</t>
         </is>
       </c>
       <c r="C155" s="19" t="inlineStr">
         <is>
-          <t>api-versioning-documentation-and-evolution</t>
+          <t>static-analysis-and-linting</t>
         </is>
       </c>
       <c r="D155" s="19" t="inlineStr">
@@ -7718,12 +7686,12 @@
       </c>
       <c r="B156" s="19" t="inlineStr">
         <is>
-          <t>apis-data-and-persistence-for-engineers</t>
+          <t>quality-assurance-and-verification</t>
         </is>
       </c>
       <c r="C156" s="19" t="inlineStr">
         <is>
-          <t>data-formats-and-serialization</t>
+          <t>software-metrics</t>
         </is>
       </c>
       <c r="D156" s="19" t="inlineStr">
@@ -7740,12 +7708,12 @@
       </c>
       <c r="B157" s="19" t="inlineStr">
         <is>
-          <t>apis-data-and-persistence-for-engineers</t>
+          <t>quality-assurance-and-verification</t>
         </is>
       </c>
       <c r="C157" s="19" t="inlineStr">
         <is>
-          <t>relational-databases-and-sql-for-developers</t>
+          <t>defect-management-and-root-cause-analysis</t>
         </is>
       </c>
       <c r="D157" s="19" t="inlineStr">
@@ -7762,12 +7730,12 @@
       </c>
       <c r="B158" s="19" t="inlineStr">
         <is>
-          <t>apis-data-and-persistence-for-engineers</t>
+          <t>quality-assurance-and-verification</t>
         </is>
       </c>
       <c r="C158" s="19" t="inlineStr">
         <is>
-          <t>transactions-and-data-integrity</t>
+          <t>reliability-and-availability-basics</t>
         </is>
       </c>
       <c r="D158" s="19" t="inlineStr">
@@ -7784,12 +7752,12 @@
       </c>
       <c r="B159" s="19" t="inlineStr">
         <is>
-          <t>apis-data-and-persistence-for-engineers</t>
+          <t>quality-assurance-and-verification</t>
         </is>
       </c>
       <c r="C159" s="19" t="inlineStr">
         <is>
-          <t>nosql-and-choosing-a-data-store</t>
+          <t>formal-specification-and-verification-an-introduction</t>
         </is>
       </c>
       <c r="D159" s="19" t="inlineStr">
@@ -7806,12 +7774,12 @@
       </c>
       <c r="B160" s="19" t="inlineStr">
         <is>
-          <t>apis-data-and-persistence-for-engineers</t>
+          <t>quality-assurance-and-verification</t>
         </is>
       </c>
       <c r="C160" s="19" t="inlineStr">
         <is>
-          <t>object-relational-mapping-and-data-access-layers</t>
+          <t>safety-critical-software</t>
         </is>
       </c>
       <c r="D160" s="19" t="inlineStr">
@@ -7828,12 +7796,12 @@
       </c>
       <c r="B161" s="19" t="inlineStr">
         <is>
-          <t>apis-data-and-persistence-for-engineers</t>
+          <t>quality-assurance-and-verification</t>
         </is>
       </c>
       <c r="C161" s="19" t="inlineStr">
         <is>
-          <t>caching-basics</t>
+          <t>learning-from-failures</t>
         </is>
       </c>
       <c r="D161" s="19" t="inlineStr">
@@ -7855,7 +7823,7 @@
       </c>
       <c r="C162" s="19" t="inlineStr">
         <is>
-          <t>concurrency-in-application-code</t>
+          <t>what-is-an-api</t>
         </is>
       </c>
       <c r="D162" s="19" t="inlineStr">
@@ -7872,12 +7840,12 @@
       </c>
       <c r="B163" s="19" t="inlineStr">
         <is>
-          <t>software-maintenance-and-evolution</t>
+          <t>apis-data-and-persistence-for-engineers</t>
         </is>
       </c>
       <c r="C163" s="19" t="inlineStr">
         <is>
-          <t>why-software-changes</t>
+          <t>designing-rest-apis</t>
         </is>
       </c>
       <c r="D163" s="19" t="inlineStr">
@@ -7894,12 +7862,12 @@
       </c>
       <c r="B164" s="19" t="inlineStr">
         <is>
-          <t>software-maintenance-and-evolution</t>
+          <t>apis-data-and-persistence-for-engineers</t>
         </is>
       </c>
       <c r="C164" s="19" t="inlineStr">
         <is>
-          <t>the-cost-of-maintenance</t>
+          <t>api-versioning-documentation-and-evolution</t>
         </is>
       </c>
       <c r="D164" s="19" t="inlineStr">
@@ -7916,12 +7884,12 @@
       </c>
       <c r="B165" s="19" t="inlineStr">
         <is>
-          <t>software-maintenance-and-evolution</t>
+          <t>apis-data-and-persistence-for-engineers</t>
         </is>
       </c>
       <c r="C165" s="19" t="inlineStr">
         <is>
-          <t>change-impact-analysis</t>
+          <t>data-formats-and-serialization</t>
         </is>
       </c>
       <c r="D165" s="19" t="inlineStr">
@@ -7938,12 +7906,12 @@
       </c>
       <c r="B166" s="19" t="inlineStr">
         <is>
-          <t>software-maintenance-and-evolution</t>
+          <t>apis-data-and-persistence-for-engineers</t>
         </is>
       </c>
       <c r="C166" s="19" t="inlineStr">
         <is>
-          <t>reverse-engineering-and-program-comprehension</t>
+          <t>relational-databases-and-sql-for-developers</t>
         </is>
       </c>
       <c r="D166" s="19" t="inlineStr">
@@ -7960,12 +7928,12 @@
       </c>
       <c r="B167" s="19" t="inlineStr">
         <is>
-          <t>software-maintenance-and-evolution</t>
+          <t>apis-data-and-persistence-for-engineers</t>
         </is>
       </c>
       <c r="C167" s="19" t="inlineStr">
         <is>
-          <t>reengineering-and-modernization</t>
+          <t>transactions-and-data-integrity</t>
         </is>
       </c>
       <c r="D167" s="19" t="inlineStr">
@@ -7982,12 +7950,12 @@
       </c>
       <c r="B168" s="19" t="inlineStr">
         <is>
-          <t>software-maintenance-and-evolution</t>
+          <t>apis-data-and-persistence-for-engineers</t>
         </is>
       </c>
       <c r="C168" s="19" t="inlineStr">
         <is>
-          <t>software-reuse</t>
+          <t>nosql-and-choosing-a-data-store</t>
         </is>
       </c>
       <c r="D168" s="19" t="inlineStr">
@@ -8004,12 +7972,12 @@
       </c>
       <c r="B169" s="19" t="inlineStr">
         <is>
-          <t>software-maintenance-and-evolution</t>
+          <t>apis-data-and-persistence-for-engineers</t>
         </is>
       </c>
       <c r="C169" s="19" t="inlineStr">
         <is>
-          <t>software-documentation</t>
+          <t>object-relational-mapping-and-data-access-layers</t>
         </is>
       </c>
       <c r="D169" s="19" t="inlineStr">
@@ -8026,12 +7994,12 @@
       </c>
       <c r="B170" s="19" t="inlineStr">
         <is>
-          <t>software-maintenance-and-evolution</t>
+          <t>apis-data-and-persistence-for-engineers</t>
         </is>
       </c>
       <c r="C170" s="19" t="inlineStr">
         <is>
-          <t>configuration-management-and-release-management</t>
+          <t>caching-basics</t>
         </is>
       </c>
       <c r="D170" s="19" t="inlineStr">
@@ -8048,12 +8016,12 @@
       </c>
       <c r="B171" s="19" t="inlineStr">
         <is>
-          <t>software-maintenance-and-evolution</t>
+          <t>apis-data-and-persistence-for-engineers</t>
         </is>
       </c>
       <c r="C171" s="19" t="inlineStr">
         <is>
-          <t>end-of-life-and-software-sustainability</t>
+          <t>concurrency-in-application-code</t>
         </is>
       </c>
       <c r="D171" s="19" t="inlineStr">
@@ -8290,7 +8258,7 @@
       </c>
       <c r="B182" s="19" t="inlineStr">
         <is>
-          <t>secure-software-development</t>
+          <t>security-ethics-and-professional-practice</t>
         </is>
       </c>
       <c r="C182" s="19" t="inlineStr">
@@ -8312,7 +8280,7 @@
       </c>
       <c r="B183" s="19" t="inlineStr">
         <is>
-          <t>secure-software-development</t>
+          <t>security-ethics-and-professional-practice</t>
         </is>
       </c>
       <c r="C183" s="19" t="inlineStr">
@@ -8334,7 +8302,7 @@
       </c>
       <c r="B184" s="19" t="inlineStr">
         <is>
-          <t>secure-software-development</t>
+          <t>security-ethics-and-professional-practice</t>
         </is>
       </c>
       <c r="C184" s="19" t="inlineStr">
@@ -8356,7 +8324,7 @@
       </c>
       <c r="B185" s="19" t="inlineStr">
         <is>
-          <t>secure-software-development</t>
+          <t>security-ethics-and-professional-practice</t>
         </is>
       </c>
       <c r="C185" s="19" t="inlineStr">
@@ -8378,7 +8346,7 @@
       </c>
       <c r="B186" s="19" t="inlineStr">
         <is>
-          <t>secure-software-development</t>
+          <t>security-ethics-and-professional-practice</t>
         </is>
       </c>
       <c r="C186" s="19" t="inlineStr">
@@ -8400,7 +8368,7 @@
       </c>
       <c r="B187" s="19" t="inlineStr">
         <is>
-          <t>secure-software-development</t>
+          <t>security-ethics-and-professional-practice</t>
         </is>
       </c>
       <c r="C187" s="19" t="inlineStr">
@@ -8422,7 +8390,7 @@
       </c>
       <c r="B188" s="19" t="inlineStr">
         <is>
-          <t>secure-software-development</t>
+          <t>security-ethics-and-professional-practice</t>
         </is>
       </c>
       <c r="C188" s="19" t="inlineStr">
@@ -8444,7 +8412,7 @@
       </c>
       <c r="B189" s="19" t="inlineStr">
         <is>
-          <t>secure-software-development</t>
+          <t>security-ethics-and-professional-practice</t>
         </is>
       </c>
       <c r="C189" s="19" t="inlineStr">
@@ -8466,7 +8434,7 @@
       </c>
       <c r="B190" s="19" t="inlineStr">
         <is>
-          <t>secure-software-development</t>
+          <t>security-ethics-and-professional-practice</t>
         </is>
       </c>
       <c r="C190" s="19" t="inlineStr">
@@ -8488,7 +8456,7 @@
       </c>
       <c r="B191" s="19" t="inlineStr">
         <is>
-          <t>professional-practice-ethics-and-modern-engineering</t>
+          <t>security-ethics-and-professional-practice</t>
         </is>
       </c>
       <c r="C191" s="19" t="inlineStr">
@@ -8510,7 +8478,7 @@
       </c>
       <c r="B192" s="19" t="inlineStr">
         <is>
-          <t>professional-practice-ethics-and-modern-engineering</t>
+          <t>security-ethics-and-professional-practice</t>
         </is>
       </c>
       <c r="C192" s="19" t="inlineStr">
@@ -8532,7 +8500,7 @@
       </c>
       <c r="B193" s="19" t="inlineStr">
         <is>
-          <t>professional-practice-ethics-and-modern-engineering</t>
+          <t>security-ethics-and-professional-practice</t>
         </is>
       </c>
       <c r="C193" s="19" t="inlineStr">
@@ -8554,7 +8522,7 @@
       </c>
       <c r="B194" s="19" t="inlineStr">
         <is>
-          <t>professional-practice-ethics-and-modern-engineering</t>
+          <t>security-ethics-and-professional-practice</t>
         </is>
       </c>
       <c r="C194" s="19" t="inlineStr">
@@ -8576,7 +8544,7 @@
       </c>
       <c r="B195" s="19" t="inlineStr">
         <is>
-          <t>professional-practice-ethics-and-modern-engineering</t>
+          <t>security-ethics-and-professional-practice</t>
         </is>
       </c>
       <c r="C195" s="19" t="inlineStr">
@@ -8598,7 +8566,7 @@
       </c>
       <c r="B196" s="19" t="inlineStr">
         <is>
-          <t>professional-practice-ethics-and-modern-engineering</t>
+          <t>security-ethics-and-professional-practice</t>
         </is>
       </c>
       <c r="C196" s="19" t="inlineStr">
@@ -8620,7 +8588,7 @@
       </c>
       <c r="B197" s="19" t="inlineStr">
         <is>
-          <t>professional-practice-ethics-and-modern-engineering</t>
+          <t>security-ethics-and-professional-practice</t>
         </is>
       </c>
       <c r="C197" s="19" t="inlineStr">
@@ -8642,7 +8610,7 @@
       </c>
       <c r="B198" s="19" t="inlineStr">
         <is>
-          <t>professional-practice-ethics-and-modern-engineering</t>
+          <t>security-ethics-and-professional-practice</t>
         </is>
       </c>
       <c r="C198" s="19" t="inlineStr">
@@ -8664,7 +8632,7 @@
       </c>
       <c r="B199" s="19" t="inlineStr">
         <is>
-          <t>professional-practice-ethics-and-modern-engineering</t>
+          <t>security-ethics-and-professional-practice</t>
         </is>
       </c>
       <c r="C199" s="19" t="inlineStr">
@@ -8686,7 +8654,7 @@
       </c>
       <c r="B200" s="19" t="inlineStr">
         <is>
-          <t>professional-practice-ethics-and-modern-engineering</t>
+          <t>security-ethics-and-professional-practice</t>
         </is>
       </c>
       <c r="C200" s="19" t="inlineStr">
@@ -8708,7 +8676,7 @@
       </c>
       <c r="B201" s="19" t="inlineStr">
         <is>
-          <t>professional-practice-ethics-and-modern-engineering</t>
+          <t>security-ethics-and-professional-practice</t>
         </is>
       </c>
       <c r="C201" s="19" t="inlineStr">
@@ -12703,7 +12671,7 @@
       </c>
       <c r="D2" s="18" t="inlineStr">
         <is>
-          <t>1, 10</t>
+          <t>1, 9</t>
         </is>
       </c>
       <c r="E2" s="18" t="inlineStr">
@@ -12740,7 +12708,7 @@
       </c>
       <c r="D3" s="18" t="inlineStr">
         <is>
-          <t>2, 3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E3" s="18" t="inlineStr">
@@ -12777,7 +12745,7 @@
       </c>
       <c r="D4" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E4" s="18" t="inlineStr">
@@ -12814,7 +12782,7 @@
       </c>
       <c r="D5" s="18" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E5" s="18" t="inlineStr">
@@ -12851,7 +12819,7 @@
       </c>
       <c r="D6" s="18" t="inlineStr">
         <is>
-          <t>6, 9</t>
+          <t>5, 8</t>
         </is>
       </c>
       <c r="E6" s="18" t="inlineStr">
@@ -12888,7 +12856,7 @@
       </c>
       <c r="D7" s="18" t="inlineStr">
         <is>
-          <t>6, 8</t>
+          <t>5, 7</t>
         </is>
       </c>
       <c r="E7" s="18" t="inlineStr">
@@ -12925,7 +12893,7 @@
       </c>
       <c r="D8" s="18" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E8" s="18" t="inlineStr">
@@ -12962,7 +12930,7 @@
       </c>
       <c r="D9" s="18" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E9" s="18" t="inlineStr">
@@ -12999,7 +12967,7 @@
       </c>
       <c r="D10" s="18" t="inlineStr">
         <is>
-          <t>11, 9</t>
+          <t>8, 10</t>
         </is>
       </c>
       <c r="E10" s="18" t="inlineStr">
@@ -13036,7 +13004,7 @@
       </c>
       <c r="D11" s="18" t="inlineStr">
         <is>
-          <t>11, 12</t>
+          <t>10, 11</t>
         </is>
       </c>
       <c r="E11" s="18" t="inlineStr">
@@ -13073,7 +13041,7 @@
       </c>
       <c r="D12" s="18" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E12" s="18" t="inlineStr">
@@ -13110,7 +13078,7 @@
       </c>
       <c r="D13" s="18" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E13" s="18" t="inlineStr">
@@ -13147,7 +13115,7 @@
       </c>
       <c r="D14" s="18" t="inlineStr">
         <is>
-          <t>13, 14</t>
+          <t>9, 12</t>
         </is>
       </c>
       <c r="E14" s="18" t="inlineStr">
@@ -13184,7 +13152,7 @@
       </c>
       <c r="D15" s="18" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E15" s="18" t="inlineStr">
@@ -13221,7 +13189,7 @@
       </c>
       <c r="D16" s="18" t="inlineStr">
         <is>
-          <t>14, 7</t>
+          <t>6, 12</t>
         </is>
       </c>
       <c r="E16" s="18" t="inlineStr">
@@ -13258,7 +13226,7 @@
       </c>
       <c r="D17" s="18" t="inlineStr">
         <is>
-          <t>7, 15</t>
+          <t>6, 8</t>
         </is>
       </c>
       <c r="E17" s="18" t="inlineStr">
@@ -13295,7 +13263,7 @@
       </c>
       <c r="D18" s="18" t="inlineStr">
         <is>
-          <t>3, 16</t>
+          <t>2, 13</t>
         </is>
       </c>
       <c r="E18" s="18" t="inlineStr">
@@ -13332,7 +13300,7 @@
       </c>
       <c r="D19" s="18" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E19" s="18" t="inlineStr">
@@ -13369,7 +13337,7 @@
       </c>
       <c r="D20" s="18" t="inlineStr">
         <is>
-          <t>10, 18</t>
+          <t>9, 14</t>
         </is>
       </c>
       <c r="E20" s="18" t="inlineStr">
@@ -13406,7 +13374,7 @@
       </c>
       <c r="D21" s="18" t="inlineStr">
         <is>
-          <t>12, 18</t>
+          <t>11, 14</t>
         </is>
       </c>
       <c r="E21" s="18" t="inlineStr">
@@ -13443,7 +13411,7 @@
       </c>
       <c r="D22" s="18" t="inlineStr">
         <is>
-          <t>1-18</t>
+          <t>1-14</t>
         </is>
       </c>
       <c r="E22" s="18" t="inlineStr">
@@ -14540,7 +14508,7 @@
       </c>
       <c r="C3" s="18" t="inlineStr">
         <is>
-          <t>2, 3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D3" s="18" t="inlineStr">
@@ -14572,7 +14540,7 @@
       </c>
       <c r="C4" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D4" s="18" t="inlineStr">
@@ -14604,7 +14572,7 @@
       </c>
       <c r="C5" s="18" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D5" s="18" t="inlineStr">
@@ -14636,7 +14604,7 @@
       </c>
       <c r="C6" s="18" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D6" s="18" t="inlineStr">
@@ -14668,7 +14636,7 @@
       </c>
       <c r="C7" s="18" t="inlineStr">
         <is>
-          <t>6, 8</t>
+          <t>5, 7</t>
         </is>
       </c>
       <c r="D7" s="18" t="inlineStr">
@@ -14700,7 +14668,7 @@
       </c>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="D8" s="18" t="inlineStr">
@@ -14732,7 +14700,7 @@
       </c>
       <c r="C9" s="18" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D9" s="18" t="inlineStr">
@@ -14764,7 +14732,7 @@
       </c>
       <c r="C10" s="18" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D10" s="18" t="inlineStr">
@@ -14796,7 +14764,7 @@
       </c>
       <c r="C11" s="18" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D11" s="18" t="inlineStr">
@@ -14828,7 +14796,7 @@
       </c>
       <c r="C12" s="18" t="inlineStr">
         <is>
-          <t>9, 15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D12" s="18" t="inlineStr">
@@ -14860,7 +14828,7 @@
       </c>
       <c r="C13" s="18" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D13" s="18" t="inlineStr">
@@ -14892,7 +14860,7 @@
       </c>
       <c r="C14" s="18" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D14" s="18" t="inlineStr">
@@ -14924,7 +14892,7 @@
       </c>
       <c r="C15" s="18" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D15" s="18" t="inlineStr">
@@ -14956,7 +14924,7 @@
       </c>
       <c r="C16" s="18" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D16" s="18" t="inlineStr">
@@ -14988,7 +14956,7 @@
       </c>
       <c r="C17" s="18" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="D17" s="18" t="inlineStr">
@@ -15020,7 +14988,7 @@
       </c>
       <c r="C18" s="18" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D18" s="18" t="inlineStr">
@@ -15052,7 +15020,7 @@
       </c>
       <c r="C19" s="18" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D19" s="18" t="inlineStr">
@@ -15084,7 +15052,7 @@
       </c>
       <c r="C20" s="18" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="D20" s="18" t="inlineStr">
@@ -15116,7 +15084,7 @@
       </c>
       <c r="C21" s="18" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>13</t>
         </is>
       </c>
       <c r="D21" s="18" t="inlineStr">
@@ -15148,7 +15116,7 @@
       </c>
       <c r="C22" s="18" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>14</t>
         </is>
       </c>
       <c r="D22" s="18" t="inlineStr">
@@ -15180,7 +15148,7 @@
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>12, 18</t>
+          <t>11, 14</t>
         </is>
       </c>
       <c r="D23" s="18" t="inlineStr">
@@ -15212,7 +15180,7 @@
       </c>
       <c r="C24" s="18" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>14</t>
         </is>
       </c>
       <c r="D24" s="18" t="inlineStr">
@@ -15244,7 +15212,7 @@
       </c>
       <c r="C25" s="18" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>14</t>
         </is>
       </c>
       <c r="D25" s="18" t="inlineStr">
@@ -15276,7 +15244,7 @@
       </c>
       <c r="C26" s="18" t="inlineStr">
         <is>
-          <t>1-18</t>
+          <t>1-14</t>
         </is>
       </c>
       <c r="D26" s="18" t="inlineStr">

</xml_diff>